<commit_message>
recover old admin files
</commit_message>
<xml_diff>
--- a/input_data/admin_data/DOM/_clean/total-pos-DOM.xlsx
+++ b/input_data/admin_data/DOM/_clean/total-pos-DOM.xlsx
@@ -14,13 +14,14 @@
     <sheet name="2017" sheetId="6" r:id="rId8"/>
     <sheet name="2018" sheetId="7" r:id="rId9"/>
     <sheet name="2019" sheetId="8" r:id="rId10"/>
+    <sheet name="2020" sheetId="9" r:id="rId11"/>
   </sheets>
   <calcPr calcId="125725" fullCalcOnLoad="true"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2752" uniqueCount="11">
   <si>
     <t>year</t>
   </si>
@@ -4900,4 +4901,605 @@
     </row>
   </sheetData>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H29"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>2020</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2">
+        <v>10446760</v>
+      </c>
+      <c r="E2">
+        <v>71294.484375</v>
+      </c>
+      <c r="F2">
+        <v>0.7546963095664978</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>11407.5048828125</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3"/>
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3"/>
+      <c r="E3"/>
+      <c r="F3">
+        <v>0.77922630310058594</v>
+      </c>
+      <c r="G3">
+        <v>23974.827965721488</v>
+      </c>
+      <c r="H3">
+        <v>37011.5546875</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4"/>
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4"/>
+      <c r="E4"/>
+      <c r="F4">
+        <v>0.80375629663467407</v>
+      </c>
+      <c r="G4">
+        <v>50941.544589819387</v>
+      </c>
+      <c r="H4">
+        <v>66469.0546875</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5"/>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5"/>
+      <c r="E5"/>
+      <c r="F5">
+        <v>0.82828617095947266</v>
+      </c>
+      <c r="G5">
+        <v>81732.47763611222</v>
+      </c>
+      <c r="H5">
+        <v>97900.1640625</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6"/>
+      <c r="B6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6"/>
+      <c r="E6"/>
+      <c r="F6">
+        <v>0.85281610488891602</v>
+      </c>
+      <c r="G6">
+        <v>113862.68020793796</v>
+      </c>
+      <c r="H6">
+        <v>126458.671875</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7"/>
+      <c r="B7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7"/>
+      <c r="E7"/>
+      <c r="F7">
+        <v>0.8773459792137146</v>
+      </c>
+      <c r="G7">
+        <v>140312.90235729623</v>
+      </c>
+      <c r="H7">
+        <v>162303.703125</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8"/>
+      <c r="B8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8"/>
+      <c r="E8"/>
+      <c r="F8">
+        <v>0.90187591314315796</v>
+      </c>
+      <c r="G8">
+        <v>188022.90355919514</v>
+      </c>
+      <c r="H8">
+        <v>221496.9375</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9"/>
+      <c r="B9" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9"/>
+      <c r="E9"/>
+      <c r="F9">
+        <v>0.92640578746795654</v>
+      </c>
+      <c r="G9">
+        <v>257079.58142312392</v>
+      </c>
+      <c r="H9">
+        <v>304394.28125</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10"/>
+      <c r="B10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10"/>
+      <c r="E10"/>
+      <c r="F10">
+        <v>0.9509357213973999</v>
+      </c>
+      <c r="G10">
+        <v>357933.14388086973</v>
+      </c>
+      <c r="H10">
+        <v>432049.3125</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11"/>
+      <c r="B11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D11"/>
+      <c r="E11"/>
+      <c r="F11">
+        <v>0.97546559572219849</v>
+      </c>
+      <c r="G11">
+        <v>526627.92403873452</v>
+      </c>
+      <c r="H11">
+        <v>545291.1875</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12"/>
+      <c r="B12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C12" t="s">
+        <v>3</v>
+      </c>
+      <c r="D12"/>
+      <c r="E12"/>
+      <c r="F12">
+        <v>0.97791862487792969</v>
+      </c>
+      <c r="G12">
+        <v>562957.09427241236</v>
+      </c>
+      <c r="H12">
+        <v>582447.9375</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13"/>
+      <c r="B13" t="s">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>3</v>
+      </c>
+      <c r="D13"/>
+      <c r="E13"/>
+      <c r="F13">
+        <v>0.98037159442901611</v>
+      </c>
+      <c r="G13">
+        <v>600230.60513713548</v>
+      </c>
+      <c r="H13">
+        <v>626180.1875</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14"/>
+      <c r="B14" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" t="s">
+        <v>3</v>
+      </c>
+      <c r="D14"/>
+      <c r="E14"/>
+      <c r="F14">
+        <v>0.98282462358474731</v>
+      </c>
+      <c r="G14">
+        <v>648096.82530098909</v>
+      </c>
+      <c r="H14">
+        <v>677552.75</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15"/>
+      <c r="B15" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15" t="s">
+        <v>3</v>
+      </c>
+      <c r="D15"/>
+      <c r="E15"/>
+      <c r="F15">
+        <v>0.98527765274047852</v>
+      </c>
+      <c r="G15">
+        <v>704065.33219000138</v>
+      </c>
+      <c r="H15">
+        <v>746018.1875</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16"/>
+      <c r="B16" t="s">
+        <v>3</v>
+      </c>
+      <c r="C16" t="s">
+        <v>3</v>
+      </c>
+      <c r="D16"/>
+      <c r="E16"/>
+      <c r="F16">
+        <v>0.98773062229156494</v>
+      </c>
+      <c r="G16">
+        <v>780106.71358774242</v>
+      </c>
+      <c r="H16">
+        <v>835712.625</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17"/>
+      <c r="B17" t="s">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>3</v>
+      </c>
+      <c r="D17"/>
+      <c r="E17"/>
+      <c r="F17">
+        <v>0.99018365144729614</v>
+      </c>
+      <c r="G17">
+        <v>883891.71305432171</v>
+      </c>
+      <c r="H17">
+        <v>966861.25</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18"/>
+      <c r="B18" t="s">
+        <v>3</v>
+      </c>
+      <c r="C18" t="s">
+        <v>3</v>
+      </c>
+      <c r="D18"/>
+      <c r="E18"/>
+      <c r="F18">
+        <v>0.99263668060302734</v>
+      </c>
+      <c r="G18">
+        <v>1042076.8757164478</v>
+      </c>
+      <c r="H18">
+        <v>1171877.625</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19"/>
+      <c r="B19" t="s">
+        <v>3</v>
+      </c>
+      <c r="C19" t="s">
+        <v>3</v>
+      </c>
+      <c r="D19"/>
+      <c r="E19"/>
+      <c r="F19">
+        <v>0.99508965015411377</v>
+      </c>
+      <c r="G19">
+        <v>1296455.1535730099</v>
+      </c>
+      <c r="H19">
+        <v>1557325.875</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20"/>
+      <c r="B20" t="s">
+        <v>3</v>
+      </c>
+      <c r="C20" t="s">
+        <v>3</v>
+      </c>
+      <c r="D20"/>
+      <c r="E20"/>
+      <c r="F20">
+        <v>0.99754256010055542</v>
+      </c>
+      <c r="G20">
+        <v>1897008.6949209895</v>
+      </c>
+      <c r="H20">
+        <v>1953034.75</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21"/>
+      <c r="B21" t="s">
+        <v>3</v>
+      </c>
+      <c r="C21" t="s">
+        <v>3</v>
+      </c>
+      <c r="D21"/>
+      <c r="E21"/>
+      <c r="F21">
+        <v>0.99778842926025391</v>
+      </c>
+      <c r="G21">
+        <v>2020021.355530163</v>
+      </c>
+      <c r="H21">
+        <v>2086303.75</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22"/>
+      <c r="B22" t="s">
+        <v>3</v>
+      </c>
+      <c r="C22" t="s">
+        <v>3</v>
+      </c>
+      <c r="D22"/>
+      <c r="E22"/>
+      <c r="F22">
+        <v>0.99803423881530762</v>
+      </c>
+      <c r="G22">
+        <v>2139682.9344491842</v>
+      </c>
+      <c r="H22">
+        <v>2223773</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23"/>
+      <c r="B23" t="s">
+        <v>3</v>
+      </c>
+      <c r="C23" t="s">
+        <v>3</v>
+      </c>
+      <c r="D23"/>
+      <c r="E23"/>
+      <c r="F23">
+        <v>0.99827992916107178</v>
+      </c>
+      <c r="G23">
+        <v>2304565.3924370673</v>
+      </c>
+      <c r="H23">
+        <v>2404741</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24"/>
+      <c r="B24" t="s">
+        <v>3</v>
+      </c>
+      <c r="C24" t="s">
+        <v>3</v>
+      </c>
+      <c r="D24"/>
+      <c r="E24"/>
+      <c r="F24">
+        <v>0.99852567911148071</v>
+      </c>
+      <c r="G24">
+        <v>2504976.6143233851</v>
+      </c>
+      <c r="H24">
+        <v>2632877.25</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25"/>
+      <c r="B25" t="s">
+        <v>3</v>
+      </c>
+      <c r="C25" t="s">
+        <v>3</v>
+      </c>
+      <c r="D25"/>
+      <c r="E25"/>
+      <c r="F25">
+        <v>0.99877136945724487</v>
+      </c>
+      <c r="G25">
+        <v>2780276.6802427149</v>
+      </c>
+      <c r="H25">
+        <v>2958662</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26"/>
+      <c r="B26" t="s">
+        <v>3</v>
+      </c>
+      <c r="C26" t="s">
+        <v>3</v>
+      </c>
+      <c r="D26"/>
+      <c r="E26"/>
+      <c r="F26">
+        <v>0.99901711940765381</v>
+      </c>
+      <c r="G26">
+        <v>3148492.0802816632</v>
+      </c>
+      <c r="H26">
+        <v>3410978</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27"/>
+      <c r="B27" t="s">
+        <v>3</v>
+      </c>
+      <c r="C27" t="s">
+        <v>3</v>
+      </c>
+      <c r="D27"/>
+      <c r="E27"/>
+      <c r="F27">
+        <v>0.99926280975341797</v>
+      </c>
+      <c r="G27">
+        <v>3716441.1441656635</v>
+      </c>
+      <c r="H27">
+        <v>4163010.75</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28"/>
+      <c r="B28" t="s">
+        <v>3</v>
+      </c>
+      <c r="C28" t="s">
+        <v>3</v>
+      </c>
+      <c r="D28"/>
+      <c r="E28"/>
+      <c r="F28">
+        <v>0.9995085597038269</v>
+      </c>
+      <c r="G28">
+        <v>4765848.8445482701</v>
+      </c>
+      <c r="H28">
+        <v>5842013.5</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29"/>
+      <c r="B29" t="s">
+        <v>3</v>
+      </c>
+      <c r="C29" t="s">
+        <v>3</v>
+      </c>
+      <c r="D29"/>
+      <c r="E29"/>
+      <c r="F29">
+        <v>0.99975425004959106</v>
+      </c>
+      <c r="G29">
+        <v>8043884.0596928</v>
+      </c>
+      <c r="H29">
+        <v>23816546</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>